<commit_message>
docs: cập nhật bảng so sánh sau khi gỡ màn chấm bài
Hai dòng « giáo viên chấm tay » và « chấm bài cho học sinh » đổi từ CẦN GỠ
sang Đã gỡ. Sheet tài khoản giáo viên thêm hai dòng cho ô « Bài cần chấm »
và nhãn trạng thái. Việc cần làm #2 thu hẹp còn /professeur/oral; #6 đổi từ
'chấm 10 bài' sang 'báo cho 10 học sinh', vì trong app không còn đường nào
để chấm chúng.

Điểm số giữ nguyên: việc gỡ làm mã khớp với quyết định, nó không thêm năng
lực nào cho sản phẩm. Thêm khối nhật ký trên sheet Tổng quan để lần mở sau
biết bản này khác bản trước ở đâu.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/so-sanh-vivoire-fracile.xlsx
+++ b/docs/so-sanh-vivoire-fracile.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="357">
   <si>
     <t>VIVOIRE  vs  FRACILE — bảng so sánh chi tiết</t>
   </si>
@@ -129,6 +129,39 @@
     <t>Chưa kiểm chứng được — KHÔNG tính vào trung bình</t>
   </si>
   <si>
+    <t>ĐÃ ĐỔI GÌ SO VỚI BẢN TRƯỚC (cùng ngày 09/09/2026)</t>
+  </si>
+  <si>
+    <t>Gỡ /professeur/copies</t>
+  </si>
+  <si>
+    <t>Route, mục menu, PEGrading.jsx và khoá nav.grading ở cả bốn từ điển. Hai dòng « giáo viên chấm tay » và « chấm bài cho học sinh » đổi từ « CẦN GỠ » sang « Đã gỡ — có chủ đích ».</t>
+  </si>
+  <si>
+    <t>Gỡ ô « Bài cần chấm »</t>
+  </si>
+  <si>
+    <t>Trang chủ giáo viên còn hai ô. Nhãn từng dòng bài nộp đổi « Chờ chấm » → « Chưa chấm ».</t>
+  </si>
+  <si>
+    <t>Sửa một câu trên màn thi</t>
+  </si>
+  <si>
+    <t>« Còn PE chờ giáo viên chấm » → nói thẳng là tự chấm theo thang DELF ở « Kết quả thi ».</t>
+  </si>
+  <si>
+    <t>Việc cần làm #2 thu hẹp</t>
+  </si>
+  <si>
+    <t>Chỉ còn /professeur/oral. Việc #6 đổi từ « chấm 10 bài » sang « báo cho 10 học sinh », vì trong app không còn đường nào để chấm chúng nữa.</t>
+  </si>
+  <si>
+    <t>Điểm số KHÔNG đổi</t>
+  </si>
+  <si>
+    <t>Việc gỡ làm mã khớp với quyết định, nó không thêm năng lực nào cho sản phẩm — nên mọi ô điểm giữ nguyên. Chỉ cột « Trạng thái » đổi.</t>
+  </si>
+  <si>
     <t>Mục so sánh</t>
   </si>
   <si>
@@ -227,13 +260,13 @@
     <t>Có — nằm trong màn lớp học của giáo viên</t>
   </si>
   <si>
-    <t>ĐÃ QUYẾT BỎ. Nhưng màn /professeur/copies VẪN CÒN trong mã</t>
-  </si>
-  <si>
-    <t>CẦN GỠ</t>
-  </si>
-  <si>
-    <t>App.jsx:264 → PEGrading.jsx; App.jsx:265 → BaiNoiGiaoVien.jsx</t>
+    <t>ĐÃ GỠ HẲN 09/09: route, mục menu, màn hình và nhãn i18n đều đi</t>
+  </si>
+  <si>
+    <t>Đã gỡ — có chủ đích</t>
+  </si>
+  <si>
+    <t>commit « Gỡ /professeur/copies ». PEGrading.jsx xoá; check:nav 94 đạt</t>
   </si>
   <si>
     <t>Lời giải thích cho câu làm sai</t>
@@ -515,13 +548,10 @@
     <t>Có — chấm tự động và AI, giáo viên chốt</t>
   </si>
   <si>
-    <t>ĐÃ QUYẾT BỎ (học sinh tự chấm / AI chấm)</t>
-  </si>
-  <si>
-    <t>CẦN GỠ /professeur/copies</t>
-  </si>
-  <si>
-    <t>Quyết định của chủ dự án 09/09/2026. Mã vẫn còn — xem sheet « Việc cần làm »</t>
+    <t>ĐÃ GỠ (học sinh tự chấm theo grille; AI chấm chưa dựng)</t>
+  </si>
+  <si>
+    <t>Quyết định và thi hành cùng ngày 09/09/2026. Xem sheet « Tài khoản giáo viên »</t>
   </si>
   <si>
     <t>Gửi nhận xét tới một học sinh</t>
@@ -779,19 +809,39 @@
     <t>/professeur/copies</t>
   </si>
   <si>
-    <t>BỎ</t>
-  </si>
-  <si>
-    <t>VẪN CÒN TRONG MÃ</t>
-  </si>
-  <si>
-    <t>Mâu thuẫn với quyết định 09/09. Route ở App.jsx:264 → PEGrading.jsx.</t>
+    <t>ĐÃ GỠ</t>
+  </si>
+  <si>
+    <t>Không còn trong mã</t>
+  </si>
+  <si>
+    <t>Gỡ 09/09/2026: route, mục menu, PEGrading.jsx và khoá nav.grading ở cả bốn từ điển. Gỡ CẢ mục menu chứ không giấu lối vào — check:nav bắt lỗi route không ai vào được.</t>
+  </si>
+  <si>
+    <t>Ô « Bài cần chấm » trên trang chủ giáo viên</t>
+  </si>
+  <si>
+    <t>/professeur/dashboard</t>
+  </si>
+  <si>
+    <t>Con số không sai, nhưng nó đếm một việc không ai làm được nữa và tô màu cảnh báo cho nó. Danh sách « Bài nộp gần đây » ngay dưới vẫn ghi rõ bài nào chưa có điểm.</t>
+  </si>
+  <si>
+    <t>Nhãn trạng thái trên từng dòng bài nộp</t>
+  </si>
+  <si>
+    <t>ĐÃ ĐỔI CHỮ</t>
+  </si>
+  <si>
+    <t>« Chờ chấm » → « Chưa chấm » (Non noté / Not marked): mô tả trạng thái thay vì hứa một hành động sẽ không xảy ra.</t>
   </si>
   <si>
     <t>MỘT CÂU PHẢI NÓI THẲNG</t>
   </si>
   <si>
-    <t>Bỏ giáo viên chấm bài KHÔNG tự động thành « AI chấm ». Hôm nay sản phẩm không có AI nào: evaluateEssayWithAI() trả về connected:false và không nơi nào trong mã gọi tới nó. Nếu gỡ /professeur/copies TRƯỚC khi dựng AI, thì trong khoảng giữa đó bài viết của học sinh chỉ còn MỘT đường duy nhất là tự chấm theo grille. Đó có thể là lựa chọn đúng — nhưng phải là lựa chọn có ý thức, không phải hệ quả tình cờ của thứ tự làm việc.</t>
+    <t xml:space="preserve">Bỏ giáo viên chấm bài KHÔNG tự động thành « AI chấm ». Hôm nay sản phẩm không có AI nào: evaluateEssayWithAI() trả về connected:false và không nơi nào trong mã gọi tới nó.
+Việc gỡ đã làm xong TRƯỚC khi AI được dựng. Nên kể từ 09/09/2026, bài viết của học sinh chỉ còn MỘT đường duy nhất: tự chấm theo grille DELF ở màn « Kết quả thi ». Đó là lựa chọn có ý thức của chủ dự án, không phải hệ quả tình cờ — nhưng nó có hạn dùng: khoảng trống này kéo dài đúng bằng thời gian tới khi việc số 4 trong sheet « Việc cần làm » (nối AI vào grille) xong.
+Và 10 bài tự luận đã nộp trước đó giờ KHÔNG còn đường nào để được chấm trong app. Nếu có học sinh đang chờ, im lặng là câu trả lời tệ nhất trong các khả năng.</t>
   </si>
   <si>
     <t>SỐ LIỆU ĐO THẬT — không con số nào ở đây là ước lượng</t>
@@ -983,13 +1033,16 @@
     <t>1 buổi</t>
   </si>
   <si>
-    <t>Quyết dứt điểm số phận /professeur/copies và /professeur/oral</t>
-  </si>
-  <si>
-    <t>Quyết định « bỏ giáo viên chấm » hiện chỉ nằm ở câu chữ; mã vẫn còn màn chấm. Để nguyên thì bảng này và sản phẩm nói hai điều khác nhau.</t>
-  </si>
-  <si>
-    <t>App.jsx:264-265; PEGrading.jsx; BaiNoiGiaoVien.jsx</t>
+    <t>Quyết số phận /professeur/oral — màn nghe bài nói</t>
+  </si>
+  <si>
+    <t>Nửa kia của việc này đã XONG 09/09: /professeur/copies và ô « Bài cần chấm » đã gỡ. Còn lại một mình màn nghe bài nói, và nó là ranh giới thật: màn đó KHÔNG cho điểm, chỉ nghe rồi nhắn nhận xét. Bỏ hẳn vai chấm thì nên gỡ; giữ vai kèm cặp thì giữ. Đây là câu hỏi về việc bạn muốn là gì với học sinh, không phải câu hỏi kỹ thuật.</t>
+  </si>
+  <si>
+    <t>App.jsx; BaiNoiGiaoVien.jsx; navItems.js</t>
+  </si>
+  <si>
+    <t>1 buổi, sau khi quyết</t>
   </si>
   <si>
     <t>Đặt neo cho 5–10 câu đọc hiểu</t>
@@ -1028,16 +1081,16 @@
     <t>1 ngày</t>
   </si>
   <si>
-    <t>Chấm 10 bài tự luận đang treo, hoặc nói cho học sinh biết là sẽ không chấm</t>
-  </si>
-  <si>
-    <t>10 bài đã nộp, chưa bài nào được chấm. Nếu có người đang chờ thì họ chờ ở đó, và im lặng là câu trả lời tệ nhất trong ba khả năng.</t>
-  </si>
-  <si>
-    <t>submissions / openMarks</t>
-  </si>
-  <si>
-    <t>tuỳ quyết định</t>
+    <t>Nói cho 10 học sinh có bài tự luận đang treo biết chuyện gì đã xảy ra</t>
+  </si>
+  <si>
+    <t>10 bài đã nộp, chưa bài nào được chấm — và từ 09/09 KHÔNG còn đường nào trong app để chấm chúng. Việc gỡ màn chấm là đúng ý bạn, nhưng nó biến 10 người đang chờ thành 10 người sẽ chờ mãi mà không được báo. Đường thông báo đã có sẵn (chuông + dấu đã đọc), nên đây là việc viết một câu, không phải việc dựng gì.</t>
+  </si>
+  <si>
+    <t>Đường thông báo đang có; submissions</t>
+  </si>
+  <si>
+    <t>30 phút</t>
   </si>
   <si>
     <t>Bổ sung ảnh màn hình thật cho trang giới thiệu</t>
@@ -1047,9 +1100,6 @@
   </si>
   <si>
     <t>LandingPage.jsx</t>
-  </si>
-  <si>
-    <t>30 phút</t>
   </si>
   <si>
     <t>Cân nhắc KHÔNG đuổi theo: từ điển, podcast, PvP, app mobile</t>
@@ -1071,7 +1121,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1119,6 +1169,12 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1F3864"/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1204,7 +1260,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1237,6 +1293,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1252,7 +1315,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1270,7 +1333,7 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1288,20 +1351,17 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1317,7 +1377,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1660,7 +1720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2015,9 +2075,84 @@
         <v>29</v>
       </c>
     </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="16" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18"/>
+    </row>
+    <row r="29" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="18"/>
+    </row>
+    <row r="30" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+    </row>
+    <row r="31" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="18"/>
+      <c r="G31" s="18"/>
+    </row>
+    <row r="32" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="6">
     <mergeCell ref="A17:G19"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B32:G32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2045,1460 +2180,1460 @@
         <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="D2" s="19">
-        <v>2</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="F2" s="19">
-        <v>2</v>
-      </c>
-      <c r="G2" s="20" t="str">
+      <c r="B2" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="22">
+        <v>2</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="22">
+        <v>2</v>
+      </c>
+      <c r="G2" s="23" t="str">
         <f>IF(OR(D2="",F2=""),"chưa rõ",IF(F2&gt;D2,"FRACILE",IF(D2&gt;F2,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H2" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I2" s="21" t="s">
-        <v>42</v>
+      <c r="H2" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I2" s="24" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="25"/>
-      <c r="E3" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="F3" s="25">
-        <v>2</v>
-      </c>
-      <c r="G3" s="26" t="str">
+      <c r="B3" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="28"/>
+      <c r="E3" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="28">
+        <v>2</v>
+      </c>
+      <c r="G3" s="29" t="str">
         <f>IF(OR(D3="",F3=""),"chưa rõ",IF(F3&gt;D3,"FRACILE",IF(D3&gt;F3,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H3" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I3" s="27" t="s">
-        <v>46</v>
+      <c r="H3" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I3" s="30" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" s="31">
-        <v>2</v>
-      </c>
-      <c r="E4" s="30" t="s">
-        <v>49</v>
-      </c>
-      <c r="F4" s="31">
+      <c r="B4" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4" s="34">
+        <v>2</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" s="34">
         <v>0</v>
       </c>
-      <c r="G4" s="32" t="str">
+      <c r="G4" s="35" t="str">
         <f>IF(OR(D4="",F4=""),"chưa rõ",IF(F4&gt;D4,"FRACILE",IF(D4&gt;F4,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H4" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="I4" s="33" t="s">
-        <v>51</v>
+      <c r="H4" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" s="36" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="19">
-        <v>2</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" s="19">
+      <c r="B5" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="22">
+        <v>2</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="F5" s="22">
         <v>1</v>
       </c>
-      <c r="G5" s="20" t="str">
+      <c r="G5" s="23" t="str">
         <f>IF(OR(D5="",F5=""),"chưa rõ",IF(F5&gt;D5,"FRACILE",IF(D5&gt;F5,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H5" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I5" s="21" t="s">
-        <v>55</v>
+      <c r="H5" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="31">
-        <v>2</v>
-      </c>
-      <c r="E6" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="F6" s="31">
+      <c r="B6" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="34">
+        <v>2</v>
+      </c>
+      <c r="E6" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="F6" s="34">
         <v>0</v>
       </c>
-      <c r="G6" s="32" t="str">
+      <c r="G6" s="35" t="str">
         <f>IF(OR(D6="",F6=""),"chưa rõ",IF(F6&gt;D6,"FRACILE",IF(D6&gt;F6,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H6" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="I6" s="33" t="s">
-        <v>59</v>
+      <c r="H6" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" s="36" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="30" t="s">
-        <v>61</v>
-      </c>
-      <c r="D7" s="31">
-        <v>2</v>
-      </c>
-      <c r="E7" s="30" t="s">
-        <v>62</v>
-      </c>
-      <c r="F7" s="31">
+      <c r="B7" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="34">
+        <v>2</v>
+      </c>
+      <c r="E7" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" s="34">
         <v>0</v>
       </c>
-      <c r="G7" s="32" t="str">
+      <c r="G7" s="35" t="str">
         <f>IF(OR(D7="",F7=""),"chưa rõ",IF(F7&gt;D7,"FRACILE",IF(D7&gt;F7,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H7" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="I7" s="33" t="s">
-        <v>64</v>
+      <c r="H7" s="31" t="s">
+        <v>74</v>
+      </c>
+      <c r="I7" s="36" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" s="25"/>
-      <c r="E8" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="F8" s="25">
-        <v>2</v>
-      </c>
-      <c r="G8" s="26" t="str">
+      <c r="B8" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="D8" s="28"/>
+      <c r="E8" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="F8" s="28">
+        <v>2</v>
+      </c>
+      <c r="G8" s="29" t="str">
         <f>IF(OR(D8="",F8=""),"chưa rõ",IF(F8&gt;D8,"FRACILE",IF(D8&gt;F8,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H8" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I8" s="27" t="s">
-        <v>68</v>
+      <c r="H8" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I8" s="30" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="18" t="s">
+      <c r="B9" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="22">
         <v>0</v>
       </c>
-      <c r="E9" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="F9" s="19">
+      <c r="E9" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="F9" s="22">
         <v>1</v>
       </c>
-      <c r="G9" s="20" t="str">
+      <c r="G9" s="23" t="str">
         <f>IF(OR(D9="",F9=""),"chưa rõ",IF(F9&gt;D9,"FRACILE",IF(D9&gt;F9,"Vivoire","hoà")))</f>
         <v>FRACILE</v>
       </c>
-      <c r="H9" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="I9" s="21" t="s">
-        <v>72</v>
+      <c r="H9" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="I9" s="24" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="19">
-        <v>2</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="F10" s="19">
+      <c r="B10" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="D10" s="22">
+        <v>2</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="F10" s="22">
         <v>1</v>
       </c>
-      <c r="G10" s="20" t="str">
+      <c r="G10" s="23" t="str">
         <f>IF(OR(D10="",F10=""),"chưa rõ",IF(F10&gt;D10,"FRACILE",IF(D10&gt;F10,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H10" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I10" s="21" t="s">
-        <v>76</v>
+      <c r="H10" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I10" s="24" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="C11" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D11" s="25"/>
-      <c r="E11" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="F11" s="25">
-        <v>2</v>
-      </c>
-      <c r="G11" s="26" t="str">
+      <c r="B11" s="26" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D11" s="28"/>
+      <c r="E11" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="28">
+        <v>2</v>
+      </c>
+      <c r="G11" s="29" t="str">
         <f>IF(OR(D11="",F11=""),"chưa rõ",IF(F11&gt;D11,"FRACILE",IF(D11&gt;F11,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H11" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I11" s="27" t="s">
-        <v>80</v>
+      <c r="H11" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I11" s="30" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="C12" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D12" s="25"/>
-      <c r="E12" s="24" t="s">
-        <v>82</v>
-      </c>
-      <c r="F12" s="25">
-        <v>2</v>
-      </c>
-      <c r="G12" s="26" t="str">
+      <c r="B12" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="C12" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D12" s="28"/>
+      <c r="E12" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="F12" s="28">
+        <v>2</v>
+      </c>
+      <c r="G12" s="29" t="str">
         <f>IF(OR(D12="",F12=""),"chưa rõ",IF(F12&gt;D12,"FRACILE",IF(D12&gt;F12,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H12" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I12" s="27" t="s">
-        <v>83</v>
+      <c r="H12" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I12" s="30" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="C13" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D13" s="25"/>
-      <c r="E13" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="F13" s="25">
-        <v>2</v>
-      </c>
-      <c r="G13" s="26" t="str">
+      <c r="B13" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="C13" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D13" s="28"/>
+      <c r="E13" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" s="28">
+        <v>2</v>
+      </c>
+      <c r="G13" s="29" t="str">
         <f>IF(OR(D13="",F13=""),"chưa rõ",IF(F13&gt;D13,"FRACILE",IF(D13&gt;F13,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H13" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I13" s="27" t="s">
-        <v>86</v>
+      <c r="H13" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I13" s="30" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="23" t="s">
-        <v>87</v>
-      </c>
-      <c r="C14" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D14" s="25"/>
-      <c r="E14" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="F14" s="25">
-        <v>2</v>
-      </c>
-      <c r="G14" s="26" t="str">
+      <c r="B14" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" s="28"/>
+      <c r="E14" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F14" s="28">
+        <v>2</v>
+      </c>
+      <c r="G14" s="29" t="str">
         <f>IF(OR(D14="",F14=""),"chưa rõ",IF(F14&gt;D14,"FRACILE",IF(D14&gt;F14,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H14" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I14" s="27" t="s">
+      <c r="H14" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I14" s="30" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="C15" s="27" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="15" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="22" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="24" t="s">
-        <v>91</v>
-      </c>
-      <c r="F15" s="25">
-        <v>2</v>
-      </c>
-      <c r="G15" s="26" t="str">
+      <c r="D15" s="28"/>
+      <c r="E15" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="F15" s="28">
+        <v>2</v>
+      </c>
+      <c r="G15" s="29" t="str">
         <f>IF(OR(D15="",F15=""),"chưa rõ",IF(F15&gt;D15,"FRACILE",IF(D15&gt;F15,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H15" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I15" s="27" t="s">
-        <v>92</v>
+      <c r="H15" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I15" s="30" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>94</v>
-      </c>
-      <c r="D16" s="19">
-        <v>2</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>95</v>
-      </c>
-      <c r="F16" s="19">
+      <c r="B16" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="D16" s="22">
+        <v>2</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="F16" s="22">
         <v>1</v>
       </c>
-      <c r="G16" s="20" t="str">
+      <c r="G16" s="23" t="str">
         <f>IF(OR(D16="",F16=""),"chưa rõ",IF(F16&gt;D16,"FRACILE",IF(D16&gt;F16,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H16" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="I16" s="21" t="s">
-        <v>97</v>
+      <c r="H16" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="I16" s="24" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="D17" s="19">
-        <v>2</v>
-      </c>
-      <c r="E17" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="F17" s="19">
+      <c r="B17" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="D17" s="22">
+        <v>2</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="F17" s="22">
         <v>1</v>
       </c>
-      <c r="G17" s="20" t="str">
+      <c r="G17" s="23" t="str">
         <f>IF(OR(D17="",F17=""),"chưa rõ",IF(F17&gt;D17,"FRACILE",IF(D17&gt;F17,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H17" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I17" s="21" t="s">
-        <v>101</v>
+      <c r="H17" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I17" s="24" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="C18" s="24" t="s">
-        <v>103</v>
-      </c>
-      <c r="D18" s="25"/>
-      <c r="E18" s="24" t="s">
-        <v>104</v>
-      </c>
-      <c r="F18" s="25">
-        <v>2</v>
-      </c>
-      <c r="G18" s="26" t="str">
+      <c r="B18" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="C18" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="D18" s="28"/>
+      <c r="E18" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="F18" s="28">
+        <v>2</v>
+      </c>
+      <c r="G18" s="29" t="str">
         <f>IF(OR(D18="",F18=""),"chưa rõ",IF(F18&gt;D18,"FRACILE",IF(D18&gt;F18,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H18" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I18" s="27" t="s">
-        <v>105</v>
+      <c r="H18" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I18" s="30" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="29" t="s">
-        <v>106</v>
-      </c>
-      <c r="C19" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="D19" s="31">
-        <v>2</v>
-      </c>
-      <c r="E19" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="F19" s="31">
+      <c r="B19" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C19" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="D19" s="34">
+        <v>2</v>
+      </c>
+      <c r="E19" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="F19" s="34">
         <v>0</v>
       </c>
-      <c r="G19" s="32" t="str">
+      <c r="G19" s="35" t="str">
         <f>IF(OR(D19="",F19=""),"chưa rõ",IF(F19&gt;D19,"FRACILE",IF(D19&gt;F19,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H19" s="28" t="s">
-        <v>109</v>
-      </c>
-      <c r="I19" s="33" t="s">
-        <v>110</v>
+      <c r="H19" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="I19" s="36" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="20" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="29" t="s">
-        <v>111</v>
-      </c>
-      <c r="C20" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="D20" s="31">
-        <v>2</v>
-      </c>
-      <c r="E20" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="F20" s="31">
+      <c r="B20" s="32" t="s">
+        <v>122</v>
+      </c>
+      <c r="C20" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20" s="34">
+        <v>2</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="F20" s="34">
         <v>0</v>
       </c>
-      <c r="G20" s="32" t="str">
+      <c r="G20" s="35" t="str">
         <f>IF(OR(D20="",F20=""),"chưa rõ",IF(F20&gt;D20,"FRACILE",IF(D20&gt;F20,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H20" s="28" t="s">
-        <v>109</v>
-      </c>
-      <c r="I20" s="33" t="s">
-        <v>112</v>
+      <c r="H20" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="I20" s="36" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="17" t="s">
-        <v>113</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="D21" s="19">
-        <v>2</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="F21" s="19">
+      <c r="B21" s="20" t="s">
+        <v>124</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" s="22">
+        <v>2</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="F21" s="22">
         <v>1</v>
       </c>
-      <c r="G21" s="20" t="str">
+      <c r="G21" s="23" t="str">
         <f>IF(OR(D21="",F21=""),"chưa rõ",IF(F21&gt;D21,"FRACILE",IF(D21&gt;F21,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H21" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I21" s="21" t="s">
-        <v>116</v>
+      <c r="H21" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I21" s="24" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="C22" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D22" s="25"/>
-      <c r="E22" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="F22" s="25">
-        <v>2</v>
-      </c>
-      <c r="G22" s="26" t="str">
+      <c r="B22" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="C22" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D22" s="28"/>
+      <c r="E22" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="F22" s="28">
+        <v>2</v>
+      </c>
+      <c r="G22" s="29" t="str">
         <f>IF(OR(D22="",F22=""),"chưa rõ",IF(F22&gt;D22,"FRACILE",IF(D22&gt;F22,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H22" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I22" s="27" t="s">
-        <v>119</v>
+      <c r="H22" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I22" s="30" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B23" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="D23" s="19">
-        <v>2</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>122</v>
-      </c>
-      <c r="F23" s="19">
-        <v>2</v>
-      </c>
-      <c r="G23" s="20" t="str">
+      <c r="B23" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="D23" s="22">
+        <v>2</v>
+      </c>
+      <c r="E23" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="F23" s="22">
+        <v>2</v>
+      </c>
+      <c r="G23" s="23" t="str">
         <f>IF(OR(D23="",F23=""),"chưa rõ",IF(F23&gt;D23,"FRACILE",IF(D23&gt;F23,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H23" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I23" s="21" t="s">
-        <v>123</v>
+      <c r="H23" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I23" s="24" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>125</v>
-      </c>
-      <c r="D24" s="19"/>
-      <c r="E24" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="F24" s="19">
+      <c r="B24" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="D24" s="22"/>
+      <c r="E24" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="F24" s="22">
         <v>1</v>
       </c>
-      <c r="G24" s="20" t="str">
+      <c r="G24" s="23" t="str">
         <f>IF(OR(D24="",F24=""),"chưa rõ",IF(F24&gt;D24,"FRACILE",IF(D24&gt;F24,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H24" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I24" s="21" t="s">
-        <v>127</v>
+      <c r="H24" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I24" s="24" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="B25" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="C25" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D25" s="25"/>
-      <c r="E25" s="24" t="s">
-        <v>129</v>
-      </c>
-      <c r="F25" s="25">
-        <v>2</v>
-      </c>
-      <c r="G25" s="26" t="str">
+      <c r="B25" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="C25" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D25" s="28"/>
+      <c r="E25" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="F25" s="28">
+        <v>2</v>
+      </c>
+      <c r="G25" s="29" t="str">
         <f>IF(OR(D25="",F25=""),"chưa rõ",IF(F25&gt;D25,"FRACILE",IF(D25&gt;F25,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H25" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I25" s="27" t="s">
-        <v>130</v>
+      <c r="H25" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I25" s="30" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="17" t="s">
-        <v>131</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>132</v>
-      </c>
-      <c r="D26" s="19">
-        <v>2</v>
-      </c>
-      <c r="E26" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="F26" s="19">
-        <v>2</v>
-      </c>
-      <c r="G26" s="20" t="str">
+      <c r="B26" s="20" t="s">
+        <v>142</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="D26" s="22">
+        <v>2</v>
+      </c>
+      <c r="E26" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="F26" s="22">
+        <v>2</v>
+      </c>
+      <c r="G26" s="23" t="str">
         <f>IF(OR(D26="",F26=""),"chưa rõ",IF(F26&gt;D26,"FRACILE",IF(D26&gt;F26,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H26" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I26" s="21" t="s">
-        <v>134</v>
+      <c r="H26" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I26" s="24" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="B27" s="29" t="s">
-        <v>135</v>
-      </c>
-      <c r="C27" s="30" t="s">
-        <v>136</v>
-      </c>
-      <c r="D27" s="31">
-        <v>2</v>
-      </c>
-      <c r="E27" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="F27" s="31">
+      <c r="B27" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C27" s="33" t="s">
+        <v>147</v>
+      </c>
+      <c r="D27" s="34">
+        <v>2</v>
+      </c>
+      <c r="E27" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="F27" s="34">
         <v>0</v>
       </c>
-      <c r="G27" s="32" t="str">
+      <c r="G27" s="35" t="str">
         <f>IF(OR(D27="",F27=""),"chưa rõ",IF(F27&gt;D27,"FRACILE",IF(D27&gt;F27,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H27" s="28" t="s">
-        <v>109</v>
-      </c>
-      <c r="I27" s="33" t="s">
-        <v>112</v>
+      <c r="H27" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="I27" s="36" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
+      <c r="A28" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B28" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="C28" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="F28" s="19">
+      <c r="B28" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D28" s="22"/>
+      <c r="E28" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="F28" s="22">
         <v>1</v>
       </c>
-      <c r="G28" s="20" t="str">
+      <c r="G28" s="23" t="str">
         <f>IF(OR(D28="",F28=""),"chưa rõ",IF(F28&gt;D28,"FRACILE",IF(D28&gt;F28,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H28" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="I28" s="21" t="s">
-        <v>140</v>
+      <c r="H28" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="I28" s="24" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B29" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="C29" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D29" s="25"/>
-      <c r="E29" s="24" t="s">
-        <v>142</v>
-      </c>
-      <c r="F29" s="25">
-        <v>2</v>
-      </c>
-      <c r="G29" s="26" t="str">
+      <c r="B29" s="26" t="s">
+        <v>152</v>
+      </c>
+      <c r="C29" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D29" s="28"/>
+      <c r="E29" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="F29" s="28">
+        <v>2</v>
+      </c>
+      <c r="G29" s="29" t="str">
         <f>IF(OR(D29="",F29=""),"chưa rõ",IF(F29&gt;D29,"FRACILE",IF(D29&gt;F29,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H29" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="I29" s="27" t="s">
-        <v>144</v>
+      <c r="H29" s="25" t="s">
+        <v>154</v>
+      </c>
+      <c r="I29" s="30" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="22" t="s">
+      <c r="A30" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B30" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="C30" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D30" s="25"/>
-      <c r="E30" s="24" t="s">
-        <v>146</v>
-      </c>
-      <c r="F30" s="25">
-        <v>2</v>
-      </c>
-      <c r="G30" s="26" t="str">
+      <c r="B30" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D30" s="28"/>
+      <c r="E30" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="F30" s="28">
+        <v>2</v>
+      </c>
+      <c r="G30" s="29" t="str">
         <f>IF(OR(D30="",F30=""),"chưa rõ",IF(F30&gt;D30,"FRACILE",IF(D30&gt;F30,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H30" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="I30" s="27" t="s">
-        <v>147</v>
+      <c r="H30" s="25" t="s">
+        <v>154</v>
+      </c>
+      <c r="I30" s="30" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="22" t="s">
+      <c r="A31" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="C31" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D31" s="25"/>
-      <c r="E31" s="24" t="s">
-        <v>149</v>
-      </c>
-      <c r="F31" s="25">
-        <v>2</v>
-      </c>
-      <c r="G31" s="26" t="str">
+      <c r="B31" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="C31" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" s="28"/>
+      <c r="E31" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="F31" s="28">
+        <v>2</v>
+      </c>
+      <c r="G31" s="29" t="str">
         <f>IF(OR(D31="",F31=""),"chưa rõ",IF(F31&gt;D31,"FRACILE",IF(D31&gt;F31,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H31" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="I31" s="27" t="s">
-        <v>150</v>
+      <c r="H31" s="25" t="s">
+        <v>154</v>
+      </c>
+      <c r="I31" s="30" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="32" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B32" s="23" t="s">
-        <v>151</v>
-      </c>
-      <c r="C32" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D32" s="25"/>
-      <c r="E32" s="24" t="s">
-        <v>152</v>
-      </c>
-      <c r="F32" s="25">
-        <v>2</v>
-      </c>
-      <c r="G32" s="26" t="str">
+      <c r="B32" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="C32" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D32" s="28"/>
+      <c r="E32" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="F32" s="28">
+        <v>2</v>
+      </c>
+      <c r="G32" s="29" t="str">
         <f>IF(OR(D32="",F32=""),"chưa rõ",IF(F32&gt;D32,"FRACILE",IF(D32&gt;F32,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H32" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="I32" s="27" t="s">
-        <v>153</v>
+      <c r="H32" s="25" t="s">
+        <v>154</v>
+      </c>
+      <c r="I32" s="30" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="33" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="16" t="s">
+      <c r="A33" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="17" t="s">
-        <v>154</v>
-      </c>
-      <c r="C33" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="D33" s="19">
-        <v>2</v>
-      </c>
-      <c r="E33" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="F33" s="19">
-        <v>2</v>
-      </c>
-      <c r="G33" s="20" t="str">
+      <c r="B33" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="D33" s="22">
+        <v>2</v>
+      </c>
+      <c r="E33" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="F33" s="22">
+        <v>2</v>
+      </c>
+      <c r="G33" s="23" t="str">
         <f>IF(OR(D33="",F33=""),"chưa rõ",IF(F33&gt;D33,"FRACILE",IF(D33&gt;F33,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H33" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="I33" s="21" t="s">
-        <v>155</v>
+      <c r="H33" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="I33" s="24" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="34" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="28" t="s">
+      <c r="A34" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B34" s="29" t="s">
-        <v>156</v>
-      </c>
-      <c r="C34" s="30" t="s">
-        <v>157</v>
-      </c>
-      <c r="D34" s="31">
-        <v>2</v>
-      </c>
-      <c r="E34" s="30" t="s">
-        <v>158</v>
-      </c>
-      <c r="F34" s="31">
+      <c r="B34" s="32" t="s">
+        <v>167</v>
+      </c>
+      <c r="C34" s="33" t="s">
+        <v>168</v>
+      </c>
+      <c r="D34" s="34">
+        <v>2</v>
+      </c>
+      <c r="E34" s="33" t="s">
+        <v>169</v>
+      </c>
+      <c r="F34" s="34">
         <v>0</v>
       </c>
-      <c r="G34" s="32" t="str">
+      <c r="G34" s="35" t="str">
         <f>IF(OR(D34="",F34=""),"chưa rõ",IF(F34&gt;D34,"FRACILE",IF(D34&gt;F34,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H34" s="28" t="s">
-        <v>159</v>
-      </c>
-      <c r="I34" s="33" t="s">
-        <v>160</v>
+      <c r="H34" s="31" t="s">
+        <v>74</v>
+      </c>
+      <c r="I34" s="36" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="35" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
+      <c r="A35" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B35" s="17" t="s">
-        <v>161</v>
-      </c>
-      <c r="C35" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="D35" s="19">
-        <v>2</v>
-      </c>
-      <c r="E35" s="18" t="s">
-        <v>162</v>
-      </c>
-      <c r="F35" s="19">
-        <v>2</v>
-      </c>
-      <c r="G35" s="20" t="str">
+      <c r="B35" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="C35" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="D35" s="22">
+        <v>2</v>
+      </c>
+      <c r="E35" s="21" t="s">
+        <v>172</v>
+      </c>
+      <c r="F35" s="22">
+        <v>2</v>
+      </c>
+      <c r="G35" s="23" t="str">
         <f>IF(OR(D35="",F35=""),"chưa rõ",IF(F35&gt;D35,"FRACILE",IF(D35&gt;F35,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H35" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="I35" s="21" t="s">
-        <v>163</v>
+      <c r="H35" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="I35" s="24" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="36" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="28" t="s">
+      <c r="A36" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="29" t="s">
-        <v>164</v>
-      </c>
-      <c r="C36" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="D36" s="31">
-        <v>2</v>
-      </c>
-      <c r="E36" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="F36" s="31">
+      <c r="B36" s="32" t="s">
+        <v>174</v>
+      </c>
+      <c r="C36" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="D36" s="34">
+        <v>2</v>
+      </c>
+      <c r="E36" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="F36" s="34">
         <v>0</v>
       </c>
-      <c r="G36" s="32" t="str">
+      <c r="G36" s="35" t="str">
         <f>IF(OR(D36="",F36=""),"chưa rõ",IF(F36&gt;D36,"FRACILE",IF(D36&gt;F36,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H36" s="28" t="s">
-        <v>109</v>
-      </c>
-      <c r="I36" s="33" t="s">
-        <v>112</v>
+      <c r="H36" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="I36" s="36" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="s">
+      <c r="A37" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B37" s="17" t="s">
-        <v>165</v>
-      </c>
-      <c r="C37" s="18" t="s">
-        <v>166</v>
-      </c>
-      <c r="D37" s="19">
-        <v>2</v>
-      </c>
-      <c r="E37" s="18" t="s">
-        <v>167</v>
-      </c>
-      <c r="F37" s="19">
+      <c r="B37" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>176</v>
+      </c>
+      <c r="D37" s="22">
+        <v>2</v>
+      </c>
+      <c r="E37" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="F37" s="22">
         <v>1</v>
       </c>
-      <c r="G37" s="20" t="str">
+      <c r="G37" s="23" t="str">
         <f>IF(OR(D37="",F37=""),"chưa rõ",IF(F37&gt;D37,"FRACILE",IF(D37&gt;F37,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H37" s="16" t="s">
-        <v>168</v>
-      </c>
-      <c r="I37" s="21" t="s">
-        <v>169</v>
+      <c r="H37" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="I37" s="24" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="16" t="s">
+      <c r="A38" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B38" s="17" t="s">
-        <v>170</v>
-      </c>
-      <c r="C38" s="18" t="s">
-        <v>103</v>
-      </c>
-      <c r="D38" s="19"/>
-      <c r="E38" s="18" t="s">
-        <v>171</v>
-      </c>
-      <c r="F38" s="19">
+      <c r="B38" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="D38" s="22"/>
+      <c r="E38" s="21" t="s">
+        <v>181</v>
+      </c>
+      <c r="F38" s="22">
         <v>1</v>
       </c>
-      <c r="G38" s="20" t="str">
+      <c r="G38" s="23" t="str">
         <f>IF(OR(D38="",F38=""),"chưa rõ",IF(F38&gt;D38,"FRACILE",IF(D38&gt;F38,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H38" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I38" s="21" t="s">
-        <v>172</v>
+      <c r="H38" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I38" s="24" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="39" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="16" t="s">
+      <c r="A39" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B39" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="C39" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="D39" s="19">
-        <v>2</v>
-      </c>
-      <c r="E39" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="F39" s="19">
-        <v>2</v>
-      </c>
-      <c r="G39" s="20" t="str">
+      <c r="B39" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="C39" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="D39" s="22">
+        <v>2</v>
+      </c>
+      <c r="E39" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="F39" s="22">
+        <v>2</v>
+      </c>
+      <c r="G39" s="23" t="str">
         <f>IF(OR(D39="",F39=""),"chưa rõ",IF(F39&gt;D39,"FRACILE",IF(D39&gt;F39,"Vivoire","hoà")))</f>
         <v>hoà</v>
       </c>
-      <c r="H39" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I39" s="21" t="s">
-        <v>174</v>
+      <c r="H39" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I39" s="24" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="40" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="28" t="s">
+      <c r="A40" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B40" s="29" t="s">
-        <v>175</v>
-      </c>
-      <c r="C40" s="30" t="s">
-        <v>176</v>
-      </c>
-      <c r="D40" s="31">
-        <v>2</v>
-      </c>
-      <c r="E40" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="F40" s="31">
+      <c r="B40" s="32" t="s">
+        <v>185</v>
+      </c>
+      <c r="C40" s="33" t="s">
+        <v>186</v>
+      </c>
+      <c r="D40" s="34">
+        <v>2</v>
+      </c>
+      <c r="E40" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="F40" s="34">
         <v>0</v>
       </c>
-      <c r="G40" s="32" t="str">
+      <c r="G40" s="35" t="str">
         <f>IF(OR(D40="",F40=""),"chưa rõ",IF(F40&gt;D40,"FRACILE",IF(D40&gt;F40,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H40" s="28" t="s">
-        <v>109</v>
-      </c>
-      <c r="I40" s="33" t="s">
-        <v>112</v>
+      <c r="H40" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="I40" s="36" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="41" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="28" t="s">
+      <c r="A41" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B41" s="29" t="s">
-        <v>177</v>
-      </c>
-      <c r="C41" s="30" t="s">
-        <v>178</v>
-      </c>
-      <c r="D41" s="31">
-        <v>2</v>
-      </c>
-      <c r="E41" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="F41" s="31">
+      <c r="B41" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="C41" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="D41" s="34">
+        <v>2</v>
+      </c>
+      <c r="E41" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="F41" s="34">
         <v>0</v>
       </c>
-      <c r="G41" s="32" t="str">
+      <c r="G41" s="35" t="str">
         <f>IF(OR(D41="",F41=""),"chưa rõ",IF(F41&gt;D41,"FRACILE",IF(D41&gt;F41,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H41" s="28" t="s">
-        <v>109</v>
-      </c>
-      <c r="I41" s="33" t="s">
-        <v>112</v>
+      <c r="H41" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="I41" s="36" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="42" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="16" t="s">
+      <c r="A42" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B42" s="17" t="s">
-        <v>179</v>
-      </c>
-      <c r="C42" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="D42" s="19">
-        <v>2</v>
-      </c>
-      <c r="E42" s="18" t="s">
-        <v>180</v>
-      </c>
-      <c r="F42" s="19">
+      <c r="B42" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="C42" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="D42" s="22">
+        <v>2</v>
+      </c>
+      <c r="E42" s="21" t="s">
+        <v>190</v>
+      </c>
+      <c r="F42" s="22">
         <v>1</v>
       </c>
-      <c r="G42" s="20" t="str">
+      <c r="G42" s="23" t="str">
         <f>IF(OR(D42="",F42=""),"chưa rõ",IF(F42&gt;D42,"FRACILE",IF(D42&gt;F42,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H42" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I42" s="21" t="s">
-        <v>112</v>
+      <c r="H42" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I42" s="24" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="43" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="22" t="s">
+      <c r="A43" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B43" s="23" t="s">
-        <v>181</v>
-      </c>
-      <c r="C43" s="24" t="s">
-        <v>182</v>
-      </c>
-      <c r="D43" s="25">
+      <c r="B43" s="26" t="s">
+        <v>191</v>
+      </c>
+      <c r="C43" s="27" t="s">
+        <v>192</v>
+      </c>
+      <c r="D43" s="28">
         <v>1</v>
       </c>
-      <c r="E43" s="24" t="s">
-        <v>183</v>
-      </c>
-      <c r="F43" s="25">
-        <v>2</v>
-      </c>
-      <c r="G43" s="26" t="str">
+      <c r="E43" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="F43" s="28">
+        <v>2</v>
+      </c>
+      <c r="G43" s="29" t="str">
         <f>IF(OR(D43="",F43=""),"chưa rõ",IF(F43&gt;D43,"FRACILE",IF(D43&gt;F43,"Vivoire","hoà")))</f>
         <v>FRACILE</v>
       </c>
-      <c r="H43" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I43" s="27" t="s">
-        <v>184</v>
+      <c r="H43" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I43" s="30" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="44" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="22" t="s">
+      <c r="A44" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B44" s="23" t="s">
-        <v>185</v>
-      </c>
-      <c r="C44" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="D44" s="25"/>
-      <c r="E44" s="24" t="s">
-        <v>186</v>
-      </c>
-      <c r="F44" s="25">
-        <v>2</v>
-      </c>
-      <c r="G44" s="26" t="str">
+      <c r="B44" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="C44" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="D44" s="28"/>
+      <c r="E44" s="27" t="s">
+        <v>196</v>
+      </c>
+      <c r="F44" s="28">
+        <v>2</v>
+      </c>
+      <c r="G44" s="29" t="str">
         <f>IF(OR(D44="",F44=""),"chưa rõ",IF(F44&gt;D44,"FRACILE",IF(D44&gt;F44,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H44" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I44" s="27" t="s">
-        <v>187</v>
+      <c r="H44" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I44" s="30" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="45" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="28" t="s">
+      <c r="A45" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B45" s="29" t="s">
-        <v>188</v>
-      </c>
-      <c r="C45" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="D45" s="31">
-        <v>2</v>
-      </c>
-      <c r="E45" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="F45" s="31">
+      <c r="B45" s="32" t="s">
+        <v>198</v>
+      </c>
+      <c r="C45" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="D45" s="34">
+        <v>2</v>
+      </c>
+      <c r="E45" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="F45" s="34">
         <v>0</v>
       </c>
-      <c r="G45" s="32" t="str">
+      <c r="G45" s="35" t="str">
         <f>IF(OR(D45="",F45=""),"chưa rõ",IF(F45&gt;D45,"FRACILE",IF(D45&gt;F45,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H45" s="28" t="s">
-        <v>189</v>
-      </c>
-      <c r="I45" s="33" t="s">
-        <v>190</v>
+      <c r="H45" s="31" t="s">
+        <v>199</v>
+      </c>
+      <c r="I45" s="36" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="46" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="28" t="s">
+      <c r="A46" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B46" s="29" t="s">
-        <v>191</v>
-      </c>
-      <c r="C46" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="D46" s="31">
-        <v>2</v>
-      </c>
-      <c r="E46" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="F46" s="31">
+      <c r="B46" s="32" t="s">
+        <v>201</v>
+      </c>
+      <c r="C46" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="D46" s="34">
+        <v>2</v>
+      </c>
+      <c r="E46" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="F46" s="34">
         <v>0</v>
       </c>
-      <c r="G46" s="32" t="str">
+      <c r="G46" s="35" t="str">
         <f>IF(OR(D46="",F46=""),"chưa rõ",IF(F46&gt;D46,"FRACILE",IF(D46&gt;F46,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H46" s="28" t="s">
-        <v>189</v>
-      </c>
-      <c r="I46" s="33" t="s">
-        <v>112</v>
+      <c r="H46" s="31" t="s">
+        <v>199</v>
+      </c>
+      <c r="I46" s="36" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="47" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="28" t="s">
+      <c r="A47" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B47" s="29" t="s">
-        <v>192</v>
-      </c>
-      <c r="C47" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="D47" s="31">
-        <v>2</v>
-      </c>
-      <c r="E47" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="F47" s="31">
+      <c r="B47" s="32" t="s">
+        <v>202</v>
+      </c>
+      <c r="C47" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="D47" s="34">
+        <v>2</v>
+      </c>
+      <c r="E47" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="F47" s="34">
         <v>0</v>
       </c>
-      <c r="G47" s="32" t="str">
+      <c r="G47" s="35" t="str">
         <f>IF(OR(D47="",F47=""),"chưa rõ",IF(F47&gt;D47,"FRACILE",IF(D47&gt;F47,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H47" s="28" t="s">
-        <v>189</v>
-      </c>
-      <c r="I47" s="33" t="s">
-        <v>193</v>
+      <c r="H47" s="31" t="s">
+        <v>199</v>
+      </c>
+      <c r="I47" s="36" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="48" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="16" t="s">
+      <c r="A48" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B48" s="17" t="s">
-        <v>194</v>
-      </c>
-      <c r="C48" s="18" t="s">
-        <v>195</v>
-      </c>
-      <c r="D48" s="19">
-        <v>2</v>
-      </c>
-      <c r="E48" s="18" t="s">
-        <v>196</v>
-      </c>
-      <c r="F48" s="19">
+      <c r="B48" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="C48" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="D48" s="22">
+        <v>2</v>
+      </c>
+      <c r="E48" s="21" t="s">
+        <v>206</v>
+      </c>
+      <c r="F48" s="22">
         <v>1</v>
       </c>
-      <c r="G48" s="20" t="str">
+      <c r="G48" s="23" t="str">
         <f>IF(OR(D48="",F48=""),"chưa rõ",IF(F48&gt;D48,"FRACILE",IF(D48&gt;F48,"Vivoire","hoà")))</f>
         <v>Vivoire</v>
       </c>
-      <c r="H48" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I48" s="21" t="s">
-        <v>197</v>
+      <c r="H48" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="I48" s="24" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="49" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="22" t="s">
+      <c r="A49" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B49" s="23" t="s">
-        <v>198</v>
-      </c>
-      <c r="C49" s="24" t="s">
-        <v>199</v>
-      </c>
-      <c r="D49" s="25">
+      <c r="B49" s="26" t="s">
+        <v>208</v>
+      </c>
+      <c r="C49" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="D49" s="28">
         <v>1</v>
       </c>
-      <c r="E49" s="24" t="s">
-        <v>200</v>
-      </c>
-      <c r="F49" s="25">
-        <v>2</v>
-      </c>
-      <c r="G49" s="26" t="str">
+      <c r="E49" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="F49" s="28">
+        <v>2</v>
+      </c>
+      <c r="G49" s="29" t="str">
         <f>IF(OR(D49="",F49=""),"chưa rõ",IF(F49&gt;D49,"FRACILE",IF(D49&gt;F49,"Vivoire","hoà")))</f>
         <v>FRACILE</v>
       </c>
-      <c r="H49" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I49" s="27" t="s">
-        <v>201</v>
+      <c r="H49" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I49" s="30" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="50" ht="44" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="22" t="s">
+      <c r="A50" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B50" s="23" t="s">
-        <v>202</v>
-      </c>
-      <c r="C50" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="D50" s="25"/>
-      <c r="E50" s="24" t="s">
-        <v>203</v>
-      </c>
-      <c r="F50" s="25">
-        <v>2</v>
-      </c>
-      <c r="G50" s="26" t="str">
+      <c r="B50" s="26" t="s">
+        <v>212</v>
+      </c>
+      <c r="C50" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="D50" s="28"/>
+      <c r="E50" s="27" t="s">
+        <v>213</v>
+      </c>
+      <c r="F50" s="28">
+        <v>2</v>
+      </c>
+      <c r="G50" s="29" t="str">
         <f>IF(OR(D50="",F50=""),"chưa rõ",IF(F50&gt;D50,"FRACILE",IF(D50&gt;F50,"Vivoire","hoà")))</f>
         <v>chưa rõ</v>
       </c>
-      <c r="H50" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="I50" s="27" t="s">
-        <v>204</v>
+      <c r="H50" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I50" s="30" t="s">
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -3510,7 +3645,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -3521,13 +3656,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
-        <v>205</v>
+      <c r="A1" s="37" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3543,247 +3678,281 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
-        <v>212</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>213</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>215</v>
+      <c r="A6" s="21" t="s">
+        <v>222</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>223</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
-        <v>216</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>217</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="E7" s="18" t="s">
-        <v>218</v>
+      <c r="A7" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="21" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
-        <v>219</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>220</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>221</v>
+      <c r="A8" s="21" t="s">
+        <v>229</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>230</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>222</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>223</v>
+      <c r="A9" s="21" t="s">
+        <v>159</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>232</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="21" t="s">
+        <v>234</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>235</v>
+      </c>
+      <c r="C10" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="B10" s="18" t="s">
-        <v>225</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>226</v>
+      <c r="D10" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
-        <v>227</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>228</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>229</v>
+      <c r="A11" s="21" t="s">
+        <v>237</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>238</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="18" t="s">
-        <v>230</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>231</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>233</v>
+      <c r="A12" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>241</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D12" s="21" t="s">
+        <v>242</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
-        <v>234</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>235</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="E13" s="18" t="s">
-        <v>112</v>
+      <c r="A13" s="21" t="s">
+        <v>244</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="18" t="s">
-        <v>236</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>237</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>238</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>239</v>
+      <c r="A14" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>247</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>248</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="35" t="s">
-        <v>240</v>
-      </c>
-      <c r="B15" s="35" t="s">
-        <v>241</v>
-      </c>
-      <c r="C15" s="36" t="s">
-        <v>242</v>
-      </c>
-      <c r="D15" s="35" t="s">
-        <v>41</v>
-      </c>
-      <c r="E15" s="35" t="s">
-        <v>243</v>
+      <c r="A15" s="38" t="s">
+        <v>250</v>
+      </c>
+      <c r="B15" s="38" t="s">
+        <v>251</v>
+      </c>
+      <c r="C15" s="39" t="s">
+        <v>252</v>
+      </c>
+      <c r="D15" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" s="38" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="30" t="s">
-        <v>244</v>
-      </c>
-      <c r="B16" s="30" t="s">
-        <v>245</v>
-      </c>
-      <c r="C16" s="28" t="s">
-        <v>246</v>
-      </c>
-      <c r="D16" s="30" t="s">
-        <v>247</v>
-      </c>
-      <c r="E16" s="30" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="37" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="38" t="s">
-        <v>250</v>
-      </c>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="38"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="38"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
+      <c r="A16" s="27" t="s">
+        <v>254</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>255</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="D16" s="27" t="s">
+        <v>257</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="27" t="s">
+        <v>259</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>260</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="D17" s="27" t="s">
+        <v>257</v>
+      </c>
+      <c r="E17" s="27" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="27" t="s">
+        <v>262</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>260</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>263</v>
+      </c>
+      <c r="D18" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="27" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="40" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="18" t="s">
+        <v>266</v>
+      </c>
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="38"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="18"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="18"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E3"/>
-    <mergeCell ref="A20:E23"/>
+    <mergeCell ref="A22:E25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -3802,303 +3971,303 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
-        <v>251</v>
+      <c r="A1" s="37" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>252</v>
+        <v>268</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>253</v>
+        <v>269</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>254</v>
+        <v>270</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="39" t="s">
-        <v>256</v>
-      </c>
-      <c r="B4" s="40">
+      <c r="A4" s="41" t="s">
+        <v>272</v>
+      </c>
+      <c r="B4" s="42">
         <v>34</v>
       </c>
-      <c r="C4" s="41" t="s">
-        <v>257</v>
-      </c>
-      <c r="D4" s="42" t="s">
-        <v>258</v>
+      <c r="C4" s="43" t="s">
+        <v>273</v>
+      </c>
+      <c r="D4" s="44" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="39" t="s">
-        <v>259</v>
-      </c>
-      <c r="B5" s="40">
+      <c r="A5" s="41" t="s">
+        <v>275</v>
+      </c>
+      <c r="B5" s="42">
         <v>373</v>
       </c>
-      <c r="C5" s="41" t="s">
-        <v>260</v>
-      </c>
-      <c r="D5" s="42" t="s">
-        <v>258</v>
+      <c r="C5" s="43" t="s">
+        <v>276</v>
+      </c>
+      <c r="D5" s="44" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="39" t="s">
-        <v>261</v>
-      </c>
-      <c r="B6" s="40">
+      <c r="A6" s="41" t="s">
+        <v>277</v>
+      </c>
+      <c r="B6" s="42">
         <v>207</v>
       </c>
-      <c r="C6" s="41" t="s">
-        <v>262</v>
-      </c>
-      <c r="D6" s="42" t="s">
-        <v>258</v>
+      <c r="C6" s="43" t="s">
+        <v>278</v>
+      </c>
+      <c r="D6" s="44" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="39" t="s">
-        <v>263</v>
-      </c>
-      <c r="B7" s="40">
+      <c r="A7" s="41" t="s">
+        <v>279</v>
+      </c>
+      <c r="B7" s="42">
         <v>0</v>
       </c>
-      <c r="C7" s="41" t="s">
-        <v>264</v>
-      </c>
-      <c r="D7" s="42" t="s">
-        <v>258</v>
+      <c r="C7" s="43" t="s">
+        <v>280</v>
+      </c>
+      <c r="D7" s="44" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="39" t="s">
-        <v>265</v>
-      </c>
-      <c r="B8" s="40">
-        <v>2</v>
-      </c>
-      <c r="C8" s="41" t="s">
-        <v>266</v>
-      </c>
-      <c r="D8" s="42" t="s">
-        <v>258</v>
+      <c r="A8" s="41" t="s">
+        <v>281</v>
+      </c>
+      <c r="B8" s="42">
+        <v>2</v>
+      </c>
+      <c r="C8" s="43" t="s">
+        <v>282</v>
+      </c>
+      <c r="D8" s="44" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="39" t="s">
-        <v>267</v>
-      </c>
-      <c r="B9" s="40">
+      <c r="A9" s="41" t="s">
+        <v>283</v>
+      </c>
+      <c r="B9" s="42">
         <v>37</v>
       </c>
-      <c r="C9" s="41" t="s">
-        <v>268</v>
-      </c>
-      <c r="D9" s="42" t="s">
-        <v>258</v>
+      <c r="C9" s="43" t="s">
+        <v>284</v>
+      </c>
+      <c r="D9" s="44" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="39" t="s">
-        <v>269</v>
-      </c>
-      <c r="B10" s="40">
+      <c r="A10" s="41" t="s">
+        <v>285</v>
+      </c>
+      <c r="B10" s="42">
         <v>156</v>
       </c>
-      <c r="C10" s="41" t="s">
-        <v>270</v>
-      </c>
-      <c r="D10" s="42" t="s">
-        <v>258</v>
+      <c r="C10" s="43" t="s">
+        <v>286</v>
+      </c>
+      <c r="D10" s="44" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="39" t="s">
-        <v>271</v>
-      </c>
-      <c r="B11" s="40">
+      <c r="A11" s="41" t="s">
+        <v>287</v>
+      </c>
+      <c r="B11" s="42">
         <v>7</v>
       </c>
-      <c r="C11" s="41" t="s">
-        <v>272</v>
-      </c>
-      <c r="D11" s="42" t="s">
-        <v>258</v>
+      <c r="C11" s="43" t="s">
+        <v>288</v>
+      </c>
+      <c r="D11" s="44" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="39" t="s">
-        <v>273</v>
-      </c>
-      <c r="B12" s="40">
+      <c r="A12" s="41" t="s">
+        <v>289</v>
+      </c>
+      <c r="B12" s="42">
         <v>10</v>
       </c>
-      <c r="C12" s="41" t="s">
+      <c r="C12" s="43" t="s">
+        <v>290</v>
+      </c>
+      <c r="D12" s="44" t="s">
         <v>274</v>
       </c>
-      <c r="D12" s="42" t="s">
-        <v>258</v>
-      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="39" t="s">
-        <v>275</v>
-      </c>
-      <c r="B13" s="40">
+      <c r="A13" s="41" t="s">
+        <v>291</v>
+      </c>
+      <c r="B13" s="42">
         <v>0</v>
       </c>
-      <c r="C13" s="41" t="s">
-        <v>276</v>
-      </c>
-      <c r="D13" s="42" t="s">
-        <v>258</v>
+      <c r="C13" s="43" t="s">
+        <v>292</v>
+      </c>
+      <c r="D13" s="44" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>277</v>
-      </c>
-      <c r="B15" s="43">
+        <v>293</v>
+      </c>
+      <c r="B15" s="45">
         <f>B6/B5</f>
         <v>0.5549597855227882</v>
       </c>
-      <c r="C15" s="44" t="s">
-        <v>278</v>
+      <c r="C15" s="46" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>279</v>
-      </c>
-      <c r="B16" s="45">
+        <v>295</v>
+      </c>
+      <c r="B16" s="47">
         <f>B5-B6</f>
         <v>166</v>
       </c>
-      <c r="C16" s="44" t="s">
-        <v>280</v>
+      <c r="C16" s="46" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="37" t="s">
-        <v>281</v>
+      <c r="A19" s="40" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="20" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>252</v>
+        <v>268</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>253</v>
+        <v>269</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>282</v>
+        <v>298</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>283</v>
+        <v>299</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="B21" s="18" t="s">
-        <v>284</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>285</v>
-      </c>
-      <c r="D21" s="18" t="s">
-        <v>286</v>
+      <c r="A21" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>300</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>301</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
-        <v>287</v>
-      </c>
-      <c r="B22" s="18" t="s">
-        <v>288</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>289</v>
-      </c>
-      <c r="D22" s="18" t="s">
-        <v>286</v>
+      <c r="A22" s="19" t="s">
+        <v>303</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>304</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="16" t="s">
-        <v>290</v>
-      </c>
-      <c r="B23" s="18" t="s">
-        <v>288</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>289</v>
-      </c>
-      <c r="D23" s="18" t="s">
-        <v>286</v>
+      <c r="A23" s="19" t="s">
+        <v>306</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>304</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="B24" s="18" t="s">
-        <v>292</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>289</v>
-      </c>
-      <c r="D24" s="18" t="s">
-        <v>286</v>
+      <c r="A24" s="19" t="s">
+        <v>307</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>308</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="D24" s="21" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="36" t="s">
-        <v>293</v>
-      </c>
-      <c r="B25" s="35" t="s">
-        <v>294</v>
-      </c>
-      <c r="C25" s="35" t="s">
-        <v>295</v>
-      </c>
-      <c r="D25" s="35" t="s">
-        <v>296</v>
+      <c r="A25" s="39" t="s">
+        <v>309</v>
+      </c>
+      <c r="B25" s="38" t="s">
+        <v>310</v>
+      </c>
+      <c r="C25" s="38" t="s">
+        <v>311</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="36" t="s">
-        <v>297</v>
-      </c>
-      <c r="B26" s="35" t="s">
-        <v>298</v>
-      </c>
-      <c r="C26" s="35" t="s">
-        <v>299</v>
-      </c>
-      <c r="D26" s="35" t="s">
-        <v>296</v>
+      <c r="A26" s="39" t="s">
+        <v>313</v>
+      </c>
+      <c r="B26" s="38" t="s">
+        <v>314</v>
+      </c>
+      <c r="C26" s="38" t="s">
+        <v>315</v>
+      </c>
+      <c r="D26" s="38" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="16" t="s">
-        <v>300</v>
-      </c>
-      <c r="B27" s="18" t="s">
-        <v>301</v>
-      </c>
-      <c r="C27" s="18" t="s">
-        <v>302</v>
-      </c>
-      <c r="D27" s="18" t="s">
-        <v>303</v>
+      <c r="A27" s="19" t="s">
+        <v>316</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>317</v>
+      </c>
+      <c r="C27" s="21" t="s">
+        <v>318</v>
+      </c>
+      <c r="D27" s="21" t="s">
+        <v>319</v>
       </c>
     </row>
   </sheetData>
@@ -4120,161 +4289,161 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
-        <v>304</v>
+      <c r="A1" s="37" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>305</v>
+        <v>321</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>306</v>
+        <v>322</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>307</v>
+        <v>323</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>308</v>
+        <v>324</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>309</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="19">
+      <c r="A4" s="22">
         <v>1</v>
       </c>
-      <c r="B4" s="16" t="s">
-        <v>310</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>311</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>312</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>313</v>
+      <c r="B4" s="19" t="s">
+        <v>326</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>327</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>328</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="19">
-        <v>2</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>314</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>315</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>313</v>
+      <c r="A5" s="22">
+        <v>2</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>330</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>331</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>332</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="19">
+      <c r="A6" s="22">
         <v>3</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>317</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>319</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>320</v>
+      <c r="B6" s="19" t="s">
+        <v>334</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>335</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>336</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="19">
+      <c r="A7" s="22">
         <v>4</v>
       </c>
-      <c r="B7" s="16" t="s">
-        <v>321</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>322</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>323</v>
-      </c>
-      <c r="E7" s="18" t="s">
-        <v>324</v>
+      <c r="B7" s="19" t="s">
+        <v>338</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>339</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>340</v>
+      </c>
+      <c r="E7" s="21" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="19">
+      <c r="A8" s="22">
         <v>5</v>
       </c>
-      <c r="B8" s="16" t="s">
-        <v>325</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>328</v>
+      <c r="B8" s="19" t="s">
+        <v>342</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>343</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>344</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="9" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="19">
+      <c r="A9" s="22">
         <v>6</v>
       </c>
-      <c r="B9" s="16" t="s">
-        <v>329</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>330</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>331</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>332</v>
+      <c r="B9" s="19" t="s">
+        <v>346</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>347</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>348</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="10" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="19">
+      <c r="A10" s="22">
         <v>7</v>
       </c>
-      <c r="B10" s="16" t="s">
-        <v>333</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>334</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>335</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>336</v>
+      <c r="B10" s="19" t="s">
+        <v>350</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>351</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>352</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="11" ht="62" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="19">
+      <c r="A11" s="22">
         <v>8</v>
       </c>
-      <c r="B11" s="16" t="s">
-        <v>337</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>338</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>339</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>340</v>
+      <c r="B11" s="19" t="s">
+        <v>353</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>354</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>355</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>